<commit_message>
docs(brfss): explain evaluation metrics with plain-language examples
</commit_message>
<xml_diff>
--- a/03_Final_Result/BRFSS_2025/outputs/model-matrix-20261007/MA_TRAN_7_MODEL_BRFSS_VI.xlsx
+++ b/03_Final_Result/BRFSS_2025/outputs/model-matrix-20261007/MA_TRAN_7_MODEL_BRFSS_VI.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ma trận 7 model" sheetId="1" r:id="R6f9b9d61f340407a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Giải thích và cấu hình" sheetId="2" r:id="Rdecb31d3065d4ee6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ma trận 7 model" sheetId="1" r:id="Rf72ea8a436f44c39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Giải thích và cấu hình" sheetId="2" r:id="R0036ab5efa0d4549"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -54,7 +54,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -86,6 +86,21 @@
         <x:fgColor rgb="FFF6F8FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE5EE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F8FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -98,7 +113,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="40">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -213,6 +228,27 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1168,7 +1204,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re28738c14d3845f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb3d47f00fa648e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1277,119 +1313,119 @@
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
       <x:c r="A11" s="37" t="str">
-        <x:v>Ý nghĩa các chỉ số</x:v>
+        <x:v>Hiểu các chỉ số bằng câu hỏi</x:v>
       </x:c>
       <x:c r="B11" s="36" t="str"/>
       <x:c r="C11" s="36" t="str"/>
     </x:row>
-    <x:row r="12" ht="54" customHeight="1">
+    <x:row r="12" ht="78" customHeight="1">
       <x:c r="A12" s="39" t="str">
         <x:v>ROC-AUC</x:v>
       </x:c>
       <x:c r="B12" s="38" t="str">
-        <x:v>Đánh giá khả năng xếp một người nhãn dương cao hơn một người nhãn âm. 0,5 tương đương xếp hạng ngẫu nhiên; 1 là phân biệt hoàn hảo.</x:v>
+        <x:v>Model có thường xếp người mang nhãn dương lên trên người mang nhãn âm không? Hãy hình dung model cho mỗi người một điểm: điểm càng cao, model càng nghiêng về nhãn dương. ROC-AUC đánh giá khả năng xếp thứ tự này qua nhiều ngưỡng.</x:v>
       </x:c>
       <x:c r="C12" s="38" t="str">
-        <x:v>Không phụ thuộc một ngưỡng cố định. ROC-AUC 0,826 không có nghĩa 82,6% người được phân loại đúng.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="62" customHeight="1">
+        <x:v>LR có ROC-AUC 0,8262. Khả năng phân biệt thứ tự tốt hơn mức ngẫu nhiên 0,5. Đây KHÔNG phải “82,62% người được phân loại đúng”. Chỉ số này không cho biết riêng số ca bắt được tại ngưỡng 0,5.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="78" customHeight="1">
       <x:c r="A13" s="17" t="str">
         <x:v>AP (Average Precision)</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
-        <x:v>Tóm tắt precision khi tăng dần recall. Giúp nhìn rõ khả năng xếp hạng nhóm dương khi nhóm này ít hơn. Càng cao càng tốt khi so cùng test.</x:v>
+        <x:v>Khi lần lượt lấy thêm người từ đầu danh sách điểm cao xuống thấp, những người được lấy có thường mang nhãn dương không? AP tóm tắt việc giữ precision khi cố tìm được nhiều ca dương hơn. Càng cao càng tốt khi so trên cùng test.</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
-        <x:v>Trong CSV nguồn tên cột là pr_auc, nhưng giá trị được tính bằng Average Precision. Không gọi nó là diện tích hình thang dưới đường precision–recall. Mốc ngẫu nhiên khoảng 0,1513 trên test này.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="54" customHeight="1">
+        <x:v>LR có AP 0,4466. Đây KHÔNG phải precision 44,66% tại ngưỡng 0,5. AP nhìn nhiều mức recall; precision trong ma trận chỉ nhìn một ngưỡng. Khi lớp dương ít, AP giúp đọc rõ kết quả của lớp này. Tên pr_auc trong nguồn ở đây thực chất là Average Precision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="78" customHeight="1">
       <x:c r="A14" s="39" t="str">
         <x:v>Precision</x:v>
       </x:c>
       <x:c r="B14" s="38" t="str">
-        <x:v>Trong những người model báo dương, có bao nhiêu người thật sự mang nhãn dương? Precision=TP/(TP+FP).</x:v>
+        <x:v>Trong những người model báo dương, đúng được bao nhiêu? Nếu model đưa ra một danh sách “dương tính”, precision cho biết danh sách đó đáng tin đến mức nào. Precision thấp nghĩa là danh sách có nhiều người bị báo nhầm.</x:v>
       </x:c>
       <x:c r="C14" s="38" t="str">
-        <x:v>Ví dụ LR: báo dương 3.414 người, đúng 1.951 người, nên precision khoảng 57,15%. “Đúng” ở đây đối chiếu nhãn khảo sát.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="54" customHeight="1">
+        <x:v>LR báo dương 3.414 người, trong đó 1.951 người mang nhãn dương. Precision = 1.951/3.414 = 57,15%. Nghĩa là khoảng 57 trong mỗi 100 người được model báo dương là đúng theo nhãn khảo sát. Không có nghĩa model tìm được 57% toàn bộ ca dương.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="78" customHeight="1">
       <x:c r="A15" s="17" t="str">
         <x:v>Recall (sensitivity)</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
-        <x:v>Trong toàn bộ người mang nhãn dương, model bắt được bao nhiêu? Recall=TP/(TP+FN).</x:v>
+        <x:v>Trong toàn bộ người mang nhãn dương, model tìm được bao nhiêu? Hãy nhìn vào nhóm cần được tìm: recall cao nghĩa là bỏ sót ít người hơn trong nhóm đó. Recall không cho biết trong danh sách model báo dương có bao nhiêu người bị báo nhầm.</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
-        <x:v>Ví dụ LR: bắt 1.951 trong 10.365 ca, nên recall khoảng 18,82%. Phần còn lại bị bỏ sót ở ngưỡng 0,5.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="54" customHeight="1">
+        <x:v>Test có 10.365 người mang nhãn dương. LR bắt được 1.951, bỏ sót 8.414. Recall = 1.951/10.365 = 18,82%. Nghĩa là tìm được khoảng 19 trong mỗi 100 ca dương tại ngưỡng 0,5. Precision hỏi về người đã báo dương; recall hỏi về toàn bộ ca dương.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="72" customHeight="1">
       <x:c r="A16" s="39" t="str">
         <x:v>F1</x:v>
       </x:c>
       <x:c r="B16" s="38" t="str">
-        <x:v>Gộp precision và recall bằng trung bình điều hòa: 2×precision×recall/(precision+recall). Cả hai cùng tốt thì F1 cao.</x:v>
+        <x:v>Model có vừa báo dương tương đối đúng, vừa tìm được nhiều ca dương không? F1 gộp precision và recall thành một con số. Nếu một trong hai thấp, F1 sẽ bị kéo xuống; nó không phải trung bình cộng thông thường.</x:v>
       </x:c>
       <x:c r="C16" s="38" t="str">
-        <x:v>Không xét trực tiếp số âm đúng và không phản ánh đầy đủ chi phí báo nhầm/bỏ sót. F1 cao nhất không tự xác định model tốt nhất cho mọi mục tiêu.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="54" customHeight="1">
+        <x:v>LR có precision 57,15% nhưng recall chỉ 18,82%, nên F1 chỉ 28,32%. Công thức: F1 = 2 × precision × recall / (precision + recall). F1 không nhìn trực tiếp số âm đúng, cũng không định giá chi phí báo nhầm và bỏ sót.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="72" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Balanced accuracy</x:v>
       </x:c>
       <x:c r="B17" s="18" t="str">
-        <x:v>Cho lớp dương và lớp âm mức đóng góp bằng nhau: (recall+specificity)/2. Giúp tránh việc lớp âm đông lấn át.</x:v>
+        <x:v>Nếu cho nhóm dương và nhóm âm tiếng nói ngang nhau, model nhận đúng hai nhóm tốt đến đâu? Chỉ số này lấy trung bình tỷ lệ bắt đúng ca dương và tỷ lệ nhận đúng ca âm, dù hai nhóm đông ít khác nhau.</x:v>
       </x:c>
       <x:c r="C17" s="18" t="str">
-        <x:v>Là kết quả tại ngưỡng đang dùng. Không thay thế ROC-AUC, AP, đánh giá xác suất hoặc lợi ích lâm sàng.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="54" customHeight="1">
+        <x:v>LR nhận đúng 18,82% nhóm dương và 97,48% nhóm âm. Balanced accuracy = (18,82% + 97,48%)/2 ≈ 58,15%. Vì vậy accuracy 85,58% chưa có nghĩa model làm tốt cả hai nhóm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="78" customHeight="1">
       <x:c r="A18" s="39" t="str">
         <x:v>Accuracy</x:v>
       </x:c>
       <x:c r="B18" s="38" t="str">
-        <x:v>Trong tất cả người được đánh giá, tỷ lệ model phân loại đúng: (TP+TN)/N.</x:v>
+        <x:v>Trong tất cả mọi người, model đoán đúng được bao nhiêu? Đây là cách đếm đúng/sai tổng quát, không phân biệt lỗi đó xảy ra ở nhóm dương hay nhóm âm.</x:v>
       </x:c>
       <x:c r="C18" s="38" t="str">
-        <x:v>Dễ bị lớp âm đông chi phối. Luôn xem cùng recall, precision và tỷ lệ lớp.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="54" customHeight="1">
+        <x:v>LR đoán đúng 58.631/68.508 người, nên accuracy 85,58%. Tuy nhiên, đoán tất cả đều âm đã được khoảng 84,87% vì nhóm âm đông. Model như vậy vẫn bỏ sót toàn bộ ca dương. Luôn đọc accuracy cùng precision, recall và tỷ lệ lớp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="72" customHeight="1">
       <x:c r="A19" s="17" t="str">
         <x:v>Specificity</x:v>
       </x:c>
       <x:c r="B19" s="18" t="str">
-        <x:v>Trong những người mang nhãn âm, model nhận đúng âm được bao nhiêu? Specificity=TN/(TN+FP).</x:v>
+        <x:v>Trong những người mang nhãn âm, model nhận đúng âm được bao nhiêu? Specificity cao nghĩa là ít người trong nhóm âm bị báo nhầm thành dương.</x:v>
       </x:c>
       <x:c r="C19" s="18" t="str">
-        <x:v>Specificity cao nghĩa là ít báo nhầm trong nhóm âm. Có thể đi kèm bỏ sót nhiều người dương, như Linear SVM tại margin 0.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="62" customHeight="1">
+        <x:v>LR nhận đúng âm 56.680/58.143 người, nên specificity 97,48%. Vẫn có 1.463 người âm bị báo dương. Specificity 97,48% không có nghĩa 97,48% những người model báo dương là đúng; câu hỏi đó thuộc precision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="78" customHeight="1">
       <x:c r="A20" s="39" t="str">
         <x:v>Brier score</x:v>
       </x:c>
       <x:c r="B20" s="38" t="str">
-        <x:v>Trung bình bình phương sai lệch giữa xác suất dự đoán và nhãn 0/1. Càng thấp càng tốt khi so cùng nhãn và tập test.</x:v>
+        <x:v>Xác suất model đưa ra có lệch nhiều so với nhãn thực tế không? Model càng tự tin mà đoán sai thì bị phạt càng nhiều. Brier là trung bình bình phương sai lệch giữa xác suất và nhãn 0/1; càng thấp càng tốt khi so cùng test.</x:v>
       </x:c>
       <x:c r="C20" s="38" t="str">
-        <x:v>Đánh giá sai số xác suất, không phải thước đo thuần calibration. Linear SVM chưa đổi margin thành xác suất nên không áp dụng, không được ghi thành 0.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="54" customHeight="1">
+        <x:v>Ví dụ minh họa: dự đoán 90%, nhãn là 1 thì sai số bình phương là (0,9−1)²=0,01; nhãn là 0 thì là (0,9−0)²=0,81. LR có Brier 0,1033, không phải “sai 10,33%”. Brier không chỉ đo calibration. SVM chưa có xác suất nên không áp dụng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="72" customHeight="1">
       <x:c r="A21" s="17" t="str">
         <x:v>TP / FP / FN / TN</x:v>
       </x:c>
       <x:c r="B21" s="18" t="str">
-        <x:v>TP: nhãn dương, dự đoán dương. FP: nhãn âm, báo dương. FN: nhãn dương, báo âm. TN: nhãn âm, dự đoán âm.</x:v>
+        <x:v>TP: báo dương và đúng. FP: báo dương nhưng nhãn âm, tức báo nhầm. FN: báo âm nhưng nhãn dương, tức bỏ sót. TN: báo âm và đúng. Bốn nhóm này là nền để tính các chỉ số ở trên.</x:v>
       </x:c>
       <x:c r="C21" s="18" t="str">
-        <x:v>Bốn cột cuối trong ma trận giữ số người để đối chiếu precision/recall. TP+FN=10.365; TN+FP=58.143 cho mỗi model.</x:v>
+        <x:v>Ví dụ LR: TP=1.951, FP=1.463, FN=8.414, TN=56.680. Trong study này, “đúng” đối chiếu trạng thái tự báo cáo đã được chẩn đoán, không phải xét nghiệm xác nhận. Mỗi người thuộc đúng một nhóm, tổng là 68.508.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="28" customHeight="1">
@@ -1794,10 +1830,102 @@
       <x:c r="B59" s="28"/>
       <x:c r="C59" s="28"/>
     </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="28"/>
-      <x:c r="B60" s="28"/>
-      <x:c r="C60" s="28"/>
+    <x:row r="60" ht="28" customHeight="1">
+      <x:c r="A60" s="42" t="str">
+        <x:v>Đọc biểu đồ và so sánh model</x:v>
+      </x:c>
+      <x:c r="B60" s="41" t="str"/>
+      <x:c r="C60" s="41" t="str"/>
+    </x:row>
+    <x:row r="61" ht="64" customHeight="1">
+      <x:c r="A61" s="44" t="str">
+        <x:v>Nhớ precision / recall</x:v>
+      </x:c>
+      <x:c r="B61" s="43" t="str">
+        <x:v>Precision: “Những người mình báo dương có đúng không?” Recall: “Mình có tìm đủ những người mang nhãn dương không?” Hai câu hỏi có mẫu số khác nhau, nên một chỉ số cao không bảo đảm chỉ số kia cao.</x:v>
+      </x:c>
+      <x:c r="C61" s="43" t="str">
+        <x:v>Một model báo dương rất ít có thể đạt precision cao nhưng bỏ sót nhiều ca. Linear SVM trong study là ví dụ: precision 62,44%, recall 12,08% tại margin 0.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="64" customHeight="1">
+      <x:c r="A62" s="46" t="str">
+        <x:v>Ngưỡng quyết định</x:v>
+      </x:c>
+      <x:c r="B62" s="45" t="str">
+        <x:v>Ngưỡng giống mức điểm để model bắt đầu báo dương. Hạ ngưỡng thì nhiều người được báo dương hơn: thường tìm được thêm ca dương, nhưng cũng có thể báo nhầm thêm người âm.</x:v>
+      </x:c>
+      <x:c r="C62" s="45" t="str">
+        <x:v>Với cùng điểm dự đoán, hạ ngưỡng làm recall không giảm và specificity không tăng. Precision có thể thay đổi không đều. Study dùng ngưỡng cố định, không tối ưu ngưỡng trên test.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="64" customHeight="1">
+      <x:c r="A63" s="44" t="str">
+        <x:v>Đường ROC</x:v>
+      </x:c>
+      <x:c r="B63" s="43" t="str">
+        <x:v>Trục dọc là recall: bắt được bao nhiêu trong nhóm dương. Trục ngang là FPR: báo nhầm bao nhiêu trong nhóm âm. Mỗi điểm là kết quả ở một ngưỡng khác nhau. Gần góc trên trái thường tốt hơn.</x:v>
+      </x:c>
+      <x:c r="C63" s="43" t="str">
+        <x:v>ROC-AUC tóm tắt khả năng xếp hạng. Đường gần nhau không đủ để kết luận hai model tương đương. Muốn biết số người đúng/sai ở một ngưỡng, đọc TP/FP/FN/TN.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="64" customHeight="1">
+      <x:c r="A64" s="46" t="str">
+        <x:v>FPR (False Positive Rate)</x:v>
+      </x:c>
+      <x:c r="B64" s="45" t="str">
+        <x:v>Trong những người mang nhãn âm, có bao nhiêu người bị model báo nhầm thành dương? FPR chính là phần còn lại của specificity.</x:v>
+      </x:c>
+      <x:c r="C64" s="45" t="str">
+        <x:v>FPR = FP/(FP+TN) = 1−specificity. LR: 1.463/58.143 ≈ 2,52%. FPR không bằng 1−precision vì mẫu số khác nhau. Đây là trục ngang của biểu đồ ROC.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="64" customHeight="1">
+      <x:c r="A65" s="44" t="str">
+        <x:v>Đường precision–recall</x:v>
+      </x:c>
+      <x:c r="B65" s="43" t="str">
+        <x:v>Trục ngang là recall, trục dọc là precision. Đi về bên phải nghĩa là tìm được nhiều ca dương hơn; lên cao nghĩa là danh sách báo dương ít lẫn người âm hơn. Mỗi điểm ứng với một ngưỡng.</x:v>
+      </x:c>
+      <x:c r="C65" s="43" t="str">
+        <x:v>Đường gần phía trên thường giữ được precision tốt hơn ở cùng recall. Đường ngang khoảng 0,151 là tỷ lệ dương trong test. AP tóm tắt đường này theo Average Precision, không phải diện tích hình thang.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="64" customHeight="1">
+      <x:c r="A66" s="46" t="str">
+        <x:v>Vì sao không có model thắng mọi mặt?</x:v>
+      </x:c>
+      <x:c r="B66" s="45" t="str">
+        <x:v>LR báo dương ít hơn và precision cao hơn GNB, nhưng bỏ sót nhiều ca hơn. GNB bắt được nhiều ca hơn, đổi lại danh sách báo dương có nhiều người âm hơn. Chọn metric phải gắn với việc muốn giảm lỗi nào.</x:v>
+      </x:c>
+      <x:c r="C66" s="45" t="str">
+        <x:v>LR: bắt 1.951 ca, báo nhầm 1.463 ca. GNB: bắt 7.340 ca, báo nhầm 15.658 ca. Đây là hành vi tại ngưỡng đang dùng, chưa phải so sánh ở cùng recall/specificity hoặc bằng chứng lợi ích lâm sàng.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="64" customHeight="1">
+      <x:c r="A67" s="44" t="str">
+        <x:v>Calibration khác ROC-AUC</x:v>
+      </x:c>
+      <x:c r="B67" s="43" t="str">
+        <x:v>ROC-AUC hỏi “xếp thứ tự có tốt không?”. Calibration hỏi “con số xác suất có sát thực tế không?”. Một model có thể xếp thứ tự tốt nhưng đưa xác suất quá cao hoặc quá thấp.</x:v>
+      </x:c>
+      <x:c r="C67" s="43" t="str">
+        <x:v>Ví dụ minh họa: nếu nhiều người cùng được dự đoán 20% thì một model hiệu chỉnh tốt sẽ có tỷ lệ nhãn dương quanh 20% trong nhóm đó. Brier đánh giá sai số xác suất tổng thể, nên cần xem thêm đường calibration.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="64" customHeight="1">
+      <x:c r="A68" s="46" t="str">
+        <x:v>Nguồn định nghĩa metric</x:v>
+      </x:c>
+      <x:c r="B68" s="45" t="str">
+        <x:v>Đối chiếu tài liệu chính thức scikit-learn. Ví dụ LR và GNB lấy từ bảng kết quả trong sheet Ma trận 7 model. Hai ví dụ về xác suất 90% và nhóm 20% chỉ minh họa cách hiểu, không phải phân tích mới của study.</x:v>
+      </x:c>
+      <x:c r="C68" s="45" t="str">
+        <x:v>https://scikit-learn.org/stable/modules/model_evaluation.html
+https://scikit-learn.org/stable/modules/calibration.html
+Đối chiếu ngày 08/10/2026.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>